<commit_message>
Sync latest content workbook to site output
</commit_message>
<xml_diff>
--- a/excel/content.xlsx
+++ b/excel/content.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13545" windowHeight="12255"/>
+    <workbookView windowWidth="27945" windowHeight="11805"/>
   </bookViews>
   <sheets>
     <sheet name="works" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="994" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="372">
   <si>
     <t>id</t>
   </si>
@@ -103,7 +103,7 @@
     <t>Other</t>
   </si>
   <si>
-    <t>欧亚国家名片-中国文化邮票</t>
+    <t>“欧亚国家名片邮票”系列</t>
   </si>
   <si>
     <t>Eurasian National Calling Cards: Chinese Culture Stamps</t>
@@ -684,6 +684,9 @@
     <t>Deep Bond Between the Military and the People</t>
   </si>
   <si>
+    <t>“人民大会堂收藏”系列</t>
+  </si>
+  <si>
     <t>Great Hall of the People Collection</t>
   </si>
   <si>
@@ -714,21 +717,6 @@
     <t>/images/exhibitions/exhibition-001/2007年12月23日在中国人民军事博物馆举办“纪念毛泽东主席诞辰114周年敬临毛体书法展览”，与毛新宇在交流.webp</t>
   </si>
   <si>
-    <t>exhibition-002</t>
-  </si>
-  <si>
-    <t>敬临毛泽东主席书法作品汇报展</t>
-  </si>
-  <si>
-    <t>Report Exhibition of Calligraphy Works in Tribute to Chairman Mao</t>
-  </si>
-  <si>
-    <t>二零零八年相关作品展出。</t>
-  </si>
-  <si>
-    <t>Related works were exhibited in 2008.</t>
-  </si>
-  <si>
     <t>exhibition-003</t>
   </si>
   <si>
@@ -789,6 +777,12 @@
     <t>Mao Zedong Poetry Calligraphy Treasures Exhibition</t>
   </si>
   <si>
+    <t>青岛</t>
+  </si>
+  <si>
+    <t>Qingdao</t>
+  </si>
+  <si>
     <t>《仿毛体手抄毛泽东诗词汇报展》作品在该展展出。</t>
   </si>
   <si>
@@ -910,9 +904,6 @@
   </si>
   <si>
     <t>In July 2009, Zhang Mantang took part in the Tokyo China Calligraphy and Fine Arts Exhibition, where he won a gold award and was also given the title of China-Japan Cultural Exchange Friendship Envoy.</t>
-  </si>
-  <si>
-    <t>nan</t>
   </si>
   <si>
     <t>/images/news/news-001/cover.webp</t>
@@ -1198,7 +1189,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1209,13 +1200,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1683,28 +1667,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1713,118 +1700,115 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2188,11 +2172,13 @@
   <dimension ref="A1:R40"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
+    <col min="7" max="7" width="33.125" customWidth="1"/>
+    <col min="8" max="8" width="37.625" customWidth="1"/>
     <col min="17" max="17" width="27.5" style="1" customWidth="1"/>
     <col min="18" max="18" width="17.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27" spans="1:18">
+    <row r="1" spans="1:18">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2304,7 +2290,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" ht="67.5" spans="1:18">
+    <row r="3" ht="27" spans="1:18">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2323,12 +2309,8 @@
       <c r="F3" t="s">
         <v>32</v>
       </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>30</v>
-      </c>
+      <c r="G3"/>
+      <c r="H3"/>
       <c r="I3" t="s">
         <v>21</v>
       </c>
@@ -2360,7 +2342,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" ht="67.5" spans="1:18">
+    <row r="4" ht="27" spans="1:18">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -2416,7 +2398,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="67.5" spans="1:18">
+    <row r="5" ht="27" spans="1:18">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -2472,7 +2454,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="67.5" spans="1:18">
+    <row r="6" ht="27" spans="1:18">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -2528,7 +2510,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" ht="67.5" spans="1:18">
+    <row r="7" ht="27" spans="1:18">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -2584,7 +2566,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" ht="67.5" spans="1:18">
+    <row r="8" ht="27" spans="1:18">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -2640,7 +2622,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" ht="67.5" spans="1:18">
+    <row r="9" ht="27" spans="1:18">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -2696,7 +2678,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="67.5" spans="1:18">
+    <row r="10" ht="27" spans="1:18">
       <c r="A10" t="s">
         <v>72</v>
       </c>
@@ -2752,7 +2734,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="67.5" spans="1:18">
+    <row r="11" ht="27" spans="1:18">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -2808,7 +2790,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" ht="67.5" spans="1:18">
+    <row r="12" ht="27" spans="1:18">
       <c r="A12" t="s">
         <v>82</v>
       </c>
@@ -2864,7 +2846,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" ht="67.5" spans="1:18">
+    <row r="13" ht="27" spans="1:18">
       <c r="A13" t="s">
         <v>86</v>
       </c>
@@ -2920,7 +2902,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" ht="67.5" spans="1:18">
+    <row r="14" ht="27" spans="1:18">
       <c r="A14" t="s">
         <v>90</v>
       </c>
@@ -2976,7 +2958,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" ht="67.5" spans="1:18">
+    <row r="15" ht="27" spans="1:18">
       <c r="A15" t="s">
         <v>93</v>
       </c>
@@ -3032,7 +3014,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" ht="67.5" spans="1:18">
+    <row r="16" ht="27" spans="1:18">
       <c r="A16" t="s">
         <v>97</v>
       </c>
@@ -3088,7 +3070,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" ht="67.5" spans="1:18">
+    <row r="17" ht="27" spans="1:18">
       <c r="A17" t="s">
         <v>101</v>
       </c>
@@ -3144,7 +3126,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" ht="67.5" spans="1:18">
+    <row r="18" ht="27" spans="1:18">
       <c r="A18" t="s">
         <v>105</v>
       </c>
@@ -3200,7 +3182,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" ht="67.5" spans="1:18">
+    <row r="19" ht="27" spans="1:18">
       <c r="A19" t="s">
         <v>109</v>
       </c>
@@ -3256,7 +3238,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" ht="67.5" spans="1:18">
+    <row r="20" ht="27" spans="1:18">
       <c r="A20" t="s">
         <v>113</v>
       </c>
@@ -3312,7 +3294,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" ht="67.5" spans="1:18">
+    <row r="21" ht="40.5" spans="1:18">
       <c r="A21" t="s">
         <v>117</v>
       </c>
@@ -3368,7 +3350,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" ht="67.5" spans="1:18">
+    <row r="22" ht="40.5" spans="1:18">
       <c r="A22" t="s">
         <v>122</v>
       </c>
@@ -3424,7 +3406,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="23" ht="67.5" spans="1:18">
+    <row r="23" ht="27" spans="1:18">
       <c r="A23" t="s">
         <v>127</v>
       </c>
@@ -3480,7 +3462,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" ht="67.5" spans="1:18">
+    <row r="24" ht="27" spans="1:18">
       <c r="A24" t="s">
         <v>131</v>
       </c>
@@ -3592,7 +3574,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="26" ht="67.5" spans="1:18">
+    <row r="26" ht="40.5" spans="1:18">
       <c r="A26" t="s">
         <v>140</v>
       </c>
@@ -3648,7 +3630,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" ht="67.5" spans="1:18">
+    <row r="27" ht="40.5" spans="1:18">
       <c r="A27" t="s">
         <v>145</v>
       </c>
@@ -3704,7 +3686,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" ht="67.5" spans="1:18">
+    <row r="28" ht="27" spans="1:18">
       <c r="A28" t="s">
         <v>149</v>
       </c>
@@ -3760,7 +3742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" ht="67.5" spans="1:18">
+    <row r="29" ht="27" spans="1:18">
       <c r="A29" t="s">
         <v>153</v>
       </c>
@@ -3816,7 +3798,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" ht="67.5" spans="1:18">
+    <row r="30" ht="27" spans="1:18">
       <c r="A30" t="s">
         <v>159</v>
       </c>
@@ -3872,7 +3854,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" ht="67.5" spans="1:18">
+    <row r="31" ht="27" spans="1:18">
       <c r="A31" t="s">
         <v>162</v>
       </c>
@@ -3928,7 +3910,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" ht="67.5" spans="1:18">
+    <row r="32" ht="27" spans="1:18">
       <c r="A32" t="s">
         <v>168</v>
       </c>
@@ -3984,7 +3966,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" ht="67.5" spans="1:18">
+    <row r="33" ht="27" spans="1:18">
       <c r="A33" t="s">
         <v>171</v>
       </c>
@@ -4040,7 +4022,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" ht="67.5" spans="1:18">
+    <row r="34" ht="27" spans="1:18">
       <c r="A34" t="s">
         <v>177</v>
       </c>
@@ -4096,7 +4078,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" ht="67.5" spans="1:18">
+    <row r="35" ht="27" spans="1:18">
       <c r="A35" t="s">
         <v>181</v>
       </c>
@@ -4152,7 +4134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" ht="67.5" spans="1:18">
+    <row r="36" ht="27" spans="1:18">
       <c r="A36" t="s">
         <v>185</v>
       </c>
@@ -4208,7 +4190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" ht="67.5" spans="1:18">
+    <row r="37" ht="27" spans="1:18">
       <c r="A37" t="s">
         <v>189</v>
       </c>
@@ -4264,7 +4246,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" ht="67.5" spans="1:18">
+    <row r="38" ht="27" spans="1:18">
       <c r="A38" t="s">
         <v>193</v>
       </c>
@@ -4320,7 +4302,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" ht="67.5" spans="1:18">
+    <row r="39" ht="27" spans="1:18">
       <c r="A39" t="s">
         <v>196</v>
       </c>
@@ -4376,7 +4358,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" ht="67.5" spans="1:18">
+    <row r="40" ht="40.5" spans="1:18">
       <c r="A40" t="s">
         <v>204</v>
       </c>
@@ -4396,10 +4378,10 @@
         <v>32</v>
       </c>
       <c r="G40" t="s">
-        <v>21</v>
+        <v>207</v>
       </c>
       <c r="H40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I40" t="s">
         <v>21</v>
@@ -4426,10 +4408,10 @@
         <v>21</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -4441,8 +4423,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="7"/>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="2" t="s">
@@ -4478,63 +4460,63 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D2">
         <v>2007</v>
       </c>
       <c r="E2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D3">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>221</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>222</v>
       </c>
       <c r="G3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="H3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>225</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
@@ -4542,226 +4524,162 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B4" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="D4">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="E4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="F4" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="G4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="H4" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="I4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="J4" t="s">
-        <v>21</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="D5">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="E5" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="F5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="G5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="H5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="I5" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="J5" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C6" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D6">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>246</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>247</v>
       </c>
       <c r="G6" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="H6" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="I6" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="J6" t="s">
-        <v>244</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="B7" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="D7">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E7" t="s">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="F7" t="s">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="G7" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="H7" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="I7" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J7" t="s">
-        <v>21</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>258</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>259</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
+        <v>260</v>
+      </c>
+      <c r="D8">
+        <v>2025</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>261</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>262</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>263</v>
       </c>
       <c r="H8" t="s">
-        <v>21</v>
+        <v>264</v>
       </c>
       <c r="I8" t="s">
-        <v>21</v>
+        <v>265</v>
       </c>
       <c r="J8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" t="s">
-        <v>253</v>
-      </c>
-      <c r="B9" t="s">
-        <v>254</v>
-      </c>
-      <c r="C9" t="s">
-        <v>255</v>
-      </c>
-      <c r="D9">
-        <v>2013</v>
-      </c>
-      <c r="E9" t="s">
-        <v>212</v>
-      </c>
-      <c r="F9" t="s">
-        <v>213</v>
-      </c>
-      <c r="G9" t="s">
-        <v>256</v>
-      </c>
-      <c r="H9" t="s">
-        <v>257</v>
-      </c>
-      <c r="I9" t="s">
-        <v>258</v>
-      </c>
-      <c r="J9" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" t="s">
-        <v>260</v>
-      </c>
-      <c r="B10" t="s">
-        <v>261</v>
-      </c>
-      <c r="C10" t="s">
-        <v>262</v>
-      </c>
-      <c r="D10">
-        <v>2025</v>
-      </c>
-      <c r="E10" t="s">
-        <v>263</v>
-      </c>
-      <c r="F10" t="s">
-        <v>264</v>
-      </c>
-      <c r="G10" t="s">
-        <v>265</v>
-      </c>
-      <c r="H10" t="s">
         <v>266</v>
-      </c>
-      <c r="I10" t="s">
-        <v>267</v>
-      </c>
-      <c r="J10" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -4790,31 +4708,31 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>275</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>16</v>
@@ -4825,57 +4743,49 @@
     </row>
     <row r="2" ht="40.5" spans="1:14">
       <c r="A2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2" t="s">
         <v>278</v>
-      </c>
-      <c r="B2" t="s">
-        <v>279</v>
-      </c>
-      <c r="C2" t="s">
-        <v>280</v>
       </c>
       <c r="D2">
         <v>2009</v>
       </c>
       <c r="E2" t="s">
+        <v>279</v>
+      </c>
+      <c r="F2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2" t="s">
         <v>281</v>
       </c>
-      <c r="F2" t="s">
+      <c r="N2" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" t="s">
-        <v>283</v>
-      </c>
-      <c r="J2" t="s">
-        <v>283</v>
-      </c>
-      <c r="K2" t="s">
-        <v>283</v>
-      </c>
-      <c r="L2" t="s">
-        <v>283</v>
-      </c>
-      <c r="M2" t="s">
-        <v>284</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="3" ht="40.5" spans="1:14">
       <c r="A3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B3" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C3" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D3">
         <v>2011</v>
@@ -4884,7 +4794,7 @@
         <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="G3" t="s">
         <v>21</v>
@@ -4892,43 +4802,35 @@
       <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" t="s">
-        <v>283</v>
-      </c>
-      <c r="J3" t="s">
-        <v>283</v>
-      </c>
-      <c r="K3" t="s">
-        <v>283</v>
-      </c>
-      <c r="L3" t="s">
-        <v>283</v>
-      </c>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3"/>
+      <c r="L3"/>
       <c r="M3" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B4" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D4">
         <v>2012</v>
       </c>
       <c r="E4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="G4" t="s">
         <v>21</v>
@@ -4936,20 +4838,12 @@
       <c r="H4" t="s">
         <v>21</v>
       </c>
-      <c r="I4" t="s">
-        <v>283</v>
-      </c>
-      <c r="J4" t="s">
-        <v>283</v>
-      </c>
-      <c r="K4" t="s">
-        <v>283</v>
-      </c>
-      <c r="L4" t="s">
-        <v>283</v>
-      </c>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
       <c r="M4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>21</v>
@@ -4957,101 +4851,87 @@
     </row>
     <row r="5" ht="40.5" spans="1:14">
       <c r="A5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B5" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C5" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D5">
         <v>2016</v>
       </c>
       <c r="E5" t="s">
+        <v>298</v>
+      </c>
+      <c r="F5" t="s">
+        <v>299</v>
+      </c>
+      <c r="G5" t="s">
+        <v>300</v>
+      </c>
+      <c r="H5" t="s">
         <v>301</v>
       </c>
-      <c r="F5" t="s">
+      <c r="I5" t="s">
         <v>302</v>
       </c>
-      <c r="G5" t="s">
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5" t="s">
         <v>303</v>
       </c>
-      <c r="H5" t="s">
+      <c r="N5" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="I5" t="s">
-        <v>305</v>
-      </c>
-      <c r="J5" t="s">
-        <v>283</v>
-      </c>
-      <c r="K5" t="s">
-        <v>283</v>
-      </c>
-      <c r="L5" t="s">
-        <v>283</v>
-      </c>
-      <c r="M5" t="s">
-        <v>306</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="6" ht="175.5" spans="1:14">
       <c r="A6" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B6" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C6" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="D6">
         <v>2023</v>
       </c>
       <c r="E6" t="s">
+        <v>308</v>
+      </c>
+      <c r="F6" t="s">
+        <v>309</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6" t="s">
+        <v>310</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="F6" t="s">
-        <v>312</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" t="s">
-        <v>283</v>
-      </c>
-      <c r="J6" t="s">
-        <v>283</v>
-      </c>
-      <c r="K6" t="s">
-        <v>283</v>
-      </c>
-      <c r="L6" t="s">
-        <v>283</v>
-      </c>
-      <c r="M6" t="s">
-        <v>313</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B7" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C7" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="D7">
         <v>2024</v>
@@ -5060,7 +4940,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="G7" t="s">
         <v>21</v>
@@ -5068,131 +4948,107 @@
       <c r="H7" t="s">
         <v>21</v>
       </c>
-      <c r="I7" t="s">
-        <v>283</v>
-      </c>
-      <c r="J7" t="s">
-        <v>283</v>
-      </c>
-      <c r="K7" t="s">
-        <v>283</v>
-      </c>
-      <c r="L7" t="s">
-        <v>283</v>
-      </c>
+      <c r="I7"/>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
       <c r="M7" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B8" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C8" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="D8">
         <v>2025</v>
       </c>
       <c r="E8" t="s">
+        <v>320</v>
+      </c>
+      <c r="F8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8" t="s">
+        <v>322</v>
+      </c>
+      <c r="N8" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="F8" t="s">
-        <v>324</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" t="s">
-        <v>283</v>
-      </c>
-      <c r="J8" t="s">
-        <v>283</v>
-      </c>
-      <c r="K8" t="s">
-        <v>283</v>
-      </c>
-      <c r="L8" t="s">
-        <v>283</v>
-      </c>
-      <c r="M8" t="s">
-        <v>325</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="9" ht="135" spans="1:14">
       <c r="A9" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B9" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C9" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="D9">
         <v>2025</v>
       </c>
       <c r="E9" t="s">
+        <v>327</v>
+      </c>
+      <c r="F9" t="s">
+        <v>328</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9"/>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9" t="s">
+        <v>329</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>330</v>
-      </c>
-      <c r="F9" t="s">
-        <v>331</v>
-      </c>
-      <c r="G9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" t="s">
-        <v>283</v>
-      </c>
-      <c r="J9" t="s">
-        <v>283</v>
-      </c>
-      <c r="K9" t="s">
-        <v>283</v>
-      </c>
-      <c r="L9" t="s">
-        <v>283</v>
-      </c>
-      <c r="M9" t="s">
-        <v>332</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B10" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C10" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D10">
         <v>2026</v>
       </c>
       <c r="E10" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F10" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="G10" t="s">
         <v>21</v>
@@ -5200,20 +5056,12 @@
       <c r="H10" t="s">
         <v>21</v>
       </c>
-      <c r="I10" t="s">
-        <v>283</v>
-      </c>
-      <c r="J10" t="s">
-        <v>283</v>
-      </c>
-      <c r="K10" t="s">
-        <v>283</v>
-      </c>
-      <c r="L10" t="s">
-        <v>283</v>
-      </c>
+      <c r="I10"/>
+      <c r="J10"/>
+      <c r="K10"/>
+      <c r="L10"/>
       <c r="M10" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>21</v>
@@ -5221,43 +5069,43 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B11" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C11" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D11">
         <v>2024</v>
       </c>
       <c r="E11" t="s">
+        <v>340</v>
+      </c>
+      <c r="F11" t="s">
+        <v>341</v>
+      </c>
+      <c r="G11" t="s">
+        <v>342</v>
+      </c>
+      <c r="H11" t="s">
+        <v>301</v>
+      </c>
+      <c r="I11" t="s">
         <v>343</v>
       </c>
-      <c r="F11" t="s">
+      <c r="J11" t="s">
         <v>344</v>
       </c>
-      <c r="G11" t="s">
+      <c r="K11" t="s">
         <v>345</v>
       </c>
-      <c r="H11" t="s">
-        <v>304</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="L11" t="s">
         <v>346</v>
       </c>
-      <c r="J11" t="s">
+      <c r="M11" t="s">
         <v>347</v>
-      </c>
-      <c r="K11" t="s">
-        <v>348</v>
-      </c>
-      <c r="L11" t="s">
-        <v>349</v>
-      </c>
-      <c r="M11" t="s">
-        <v>350</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>21</v>
@@ -5265,43 +5113,41 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B12" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C12" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="D12">
         <v>2016</v>
       </c>
       <c r="E12" t="s">
+        <v>351</v>
+      </c>
+      <c r="F12" t="s">
+        <v>352</v>
+      </c>
+      <c r="G12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12"/>
+      <c r="J12" t="s">
+        <v>344</v>
+      </c>
+      <c r="K12" t="s">
+        <v>345</v>
+      </c>
+      <c r="L12" t="s">
+        <v>353</v>
+      </c>
+      <c r="M12" t="s">
         <v>354</v>
-      </c>
-      <c r="F12" t="s">
-        <v>355</v>
-      </c>
-      <c r="G12" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" t="s">
-        <v>283</v>
-      </c>
-      <c r="J12" t="s">
-        <v>347</v>
-      </c>
-      <c r="K12" t="s">
-        <v>348</v>
-      </c>
-      <c r="L12" t="s">
-        <v>356</v>
-      </c>
-      <c r="M12" t="s">
-        <v>357</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>21</v>
@@ -5309,43 +5155,37 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B13" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C13" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="D13">
         <v>2008</v>
       </c>
       <c r="E13" t="s">
+        <v>358</v>
+      </c>
+      <c r="F13" t="s">
+        <v>359</v>
+      </c>
+      <c r="G13" t="s">
+        <v>360</v>
+      </c>
+      <c r="H13" t="s">
+        <v>301</v>
+      </c>
+      <c r="I13" t="s">
         <v>361</v>
       </c>
-      <c r="F13" t="s">
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13" t="s">
         <v>362</v>
-      </c>
-      <c r="G13" t="s">
-        <v>363</v>
-      </c>
-      <c r="H13" t="s">
-        <v>304</v>
-      </c>
-      <c r="I13" t="s">
-        <v>364</v>
-      </c>
-      <c r="J13" t="s">
-        <v>283</v>
-      </c>
-      <c r="K13" t="s">
-        <v>283</v>
-      </c>
-      <c r="L13" t="s">
-        <v>283</v>
-      </c>
-      <c r="M13" t="s">
-        <v>365</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>21</v>
@@ -5353,43 +5193,37 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C14" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D14">
         <v>2011</v>
       </c>
       <c r="E14" t="s">
+        <v>366</v>
+      </c>
+      <c r="F14" t="s">
+        <v>367</v>
+      </c>
+      <c r="G14" t="s">
+        <v>368</v>
+      </c>
+      <c r="H14" t="s">
         <v>369</v>
       </c>
-      <c r="F14" t="s">
+      <c r="I14" t="s">
         <v>370</v>
       </c>
-      <c r="G14" t="s">
+      <c r="J14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14" t="s">
         <v>371</v>
-      </c>
-      <c r="H14" t="s">
-        <v>372</v>
-      </c>
-      <c r="I14" t="s">
-        <v>373</v>
-      </c>
-      <c r="J14" t="s">
-        <v>283</v>
-      </c>
-      <c r="K14" t="s">
-        <v>283</v>
-      </c>
-      <c r="L14" t="s">
-        <v>283</v>
-      </c>
-      <c r="M14" t="s">
-        <v>374</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>21</v>

</xml_diff>